<commit_message>
Updated the OT Scheduler class and improved Excel processing. All surgeries have been scheduled on time.
</commit_message>
<xml_diff>
--- a/OT_Scheduling/assets/OT preferences(1).xlsx
+++ b/OT_Scheduling/assets/OT preferences(1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhis\Workspace\backend\OT-Scheduler\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABD46D0F-D7A0-4CF7-BC45-EACAA3B29CD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCBF2EB-6CCA-496E-A54D-45ABCBB9C0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9648" yWindow="1260" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Department-OT Mapping" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
@@ -39,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="111">
   <si>
     <t>Sr No</t>
   </si>
@@ -342,31 +340,40 @@
     <t>Cath lab</t>
   </si>
   <si>
-    <t>6,7</t>
-  </si>
-  <si>
-    <t>1,3,7,11</t>
-  </si>
-  <si>
-    <t>1,11</t>
-  </si>
-  <si>
-    <t>10,11</t>
-  </si>
-  <si>
-    <t>4,7</t>
-  </si>
-  <si>
-    <t>1,3,7</t>
-  </si>
-  <si>
     <t>1,2</t>
   </si>
   <si>
-    <t>3,11</t>
-  </si>
-  <si>
     <t>Breast Oncology</t>
+  </si>
+  <si>
+    <t>5,6,7,8,11</t>
+  </si>
+  <si>
+    <t>3,4</t>
+  </si>
+  <si>
+    <t>7,9,11</t>
+  </si>
+  <si>
+    <t>7,11</t>
+  </si>
+  <si>
+    <t>7,10</t>
+  </si>
+  <si>
+    <t>8,5</t>
+  </si>
+  <si>
+    <t>6,2</t>
+  </si>
+  <si>
+    <t>10,9</t>
+  </si>
+  <si>
+    <t>7,11,9</t>
+  </si>
+  <si>
+    <t>1,2,10</t>
   </si>
 </sst>
 </file>
@@ -814,10 +821,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1">
@@ -828,7 +835,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="2">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1">
@@ -839,7 +846,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="2">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1">
@@ -949,7 +956,7 @@
         <v>14</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15" customHeight="1">
@@ -960,7 +967,7 @@
         <v>15</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15" customHeight="1">
@@ -971,7 +978,7 @@
         <v>16</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15" customHeight="1">
@@ -982,7 +989,7 @@
         <v>17</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" customHeight="1">
@@ -1004,7 +1011,7 @@
         <v>19</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" customHeight="1">
@@ -1036,8 +1043,8 @@
       <c r="B22" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="2">
-        <v>7</v>
+      <c r="C22" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15" customHeight="1">
@@ -1048,7 +1055,7 @@
         <v>23</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.4">
@@ -1059,7 +1066,7 @@
         <v>24</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.4">
@@ -1081,7 +1088,7 @@
         <v>26</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.4">
@@ -1103,7 +1110,7 @@
         <v>28</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="14.4">
@@ -1114,7 +1121,7 @@
         <v>29</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.4">
@@ -1125,7 +1132,7 @@
         <v>30</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.4">
@@ -1136,7 +1143,7 @@
         <v>31</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.4">
@@ -1147,7 +1154,7 @@
         <v>32</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="14.4">
@@ -1158,7 +1165,7 @@
         <v>33</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>